<commit_message>
save 04 03 2026
</commit_message>
<xml_diff>
--- a/3 четверть_3_Java Junior.xlsx
+++ b/3 четверть_3_Java Junior.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58007A7E-6F0A-4CE0-9CC9-8EEB8FF3F6D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A850D56F-3D03-4EB7-B7E8-23DD91207A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10875" yWindow="-18720" windowWidth="23250" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-13875" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Название 1-3" sheetId="12" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1611" uniqueCount="1398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1612" uniqueCount="1399">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -25141,6 +25141,153 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">`@Service
+public class BotMessageService {
+    public void </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>handleStart</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(Context ctx, Message message) {
+        ctx.sendMessage(message.chat.id, "Hello, I am spring-boot echo bot").exec();
+    }
+    public void </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>handleText</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Context ctx, Message message) {
+        ctx.sendMessage(message.chat.id, message.text).exec();
+    }
+}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">public class MyFirstBot {
+  static final String TOKEN = "YOUR_BOT_TOKEN_HERE";
+  public static void main(String[] args) {
+    final BotClient bot = new BotClient(TOKEN);
+    // Responding to /start command
+    bot.onMessage(filter -&gt; filter.commands("start"), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(context, message) -&gt; {
+        context.sendMessage(message.chat.id, "Welcome!").exec();
+    }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">);
+    // Echoing any incoming text
+    bot.onMessage(filter -&gt; filter.text(), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(context, message) -&gt; {
+        context.sendMessage(message.chat.id, message.text).exec();
+    }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>);</t>
+    </r>
+  </si>
+  <si>
+    <t>Лямбда-выражение</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Пояснение! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ bot.onMessage реализован с двумя аргументами. Второй аргумент должен быть лямба-выражением, либо методом референсом, который реализован где-то отдельно.</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">`@RestController
 class WebhookController {
     private final BotClient bot;
@@ -25162,7 +25309,7 @@
         <charset val="204"/>
         <scheme val="minor"/>
       </rPr>
-      <t>botService::handleStart</t>
+      <t>BotServiceMyClass::handleStart</t>
     </r>
     <r>
       <rPr>
@@ -25187,7 +25334,7 @@
         <charset val="204"/>
         <scheme val="minor"/>
       </rPr>
-      <t>botService::handleText</t>
+      <t>BotServiceMyClass::handleText</t>
     </r>
     <r>
       <rPr>
@@ -25203,163 +25350,27 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">`@Service
-public class BotMessageService {
-    public void </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>handleStart</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">(Context ctx, Message message) {
-        ctx.sendMessage(message.chat.id, "Hello, I am spring-boot echo bot").exec();
-    }
-    public void </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>handleText</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(Context ctx, Message message) {
-        ctx.sendMessage(message.chat.id, message.text).exec();
-    }
-}</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">public class MyFirstBot {
-  static final String TOKEN = "YOUR_BOT_TOKEN_HERE";
-  public static void main(String[] args) {
-    final BotClient bot = new BotClient(TOKEN);
-    // Responding to /start command
-    bot.onMessage(filter -&gt; filter.commands("start"), </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(context, message) -&gt; {
-        context.sendMessage(message.chat.id, "Welcome!").exec();
-    }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">);
-    // Echoing any incoming text
-    bot.onMessage(filter -&gt; filter.text(), </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(context, message) -&gt; {
-        context.sendMessage(message.chat.id, message.text).exec();
-    }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>);</t>
-    </r>
-  </si>
-  <si>
-    <t>Лямбда-выражение</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Пояснение! </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
- bot.onMessage реализован с двумя аргументами. Второй аргумент должен быть лямба-выражением, либо методом референсом, который реализован где-то отдельно.</t>
-    </r>
+    <t>Пример  на основе тг бота</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="74">
+  <fonts count="75">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -26270,9 +26281,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="276">
+  <cellXfs count="277">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -26283,24 +26294,30 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="56" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="56" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="54" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="54" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="54" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="53" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -26308,37 +26325,31 @@
     <xf numFmtId="49" fontId="53" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="52" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="52" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="52" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="51" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="51" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="51" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="57" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="50" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="57" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="50" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="51" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26347,7 +26358,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="50" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="51" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26359,7 +26370,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="50" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="51" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26371,7 +26382,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="50" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="51" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26380,25 +26391,25 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="50" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="51" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="50" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="51" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26407,28 +26418,28 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26449,34 +26460,34 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="49" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="50" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="56" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26491,26 +26502,50 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="48" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="49" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="48" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="49" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="48" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="49" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="48" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="49" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="47" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="48" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="48" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="48" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="48" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="48" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="56" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="61" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -26518,67 +26553,43 @@
     <xf numFmtId="49" fontId="47" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="55" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="60" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="46" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="44" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="45" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="44" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="45" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="44" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="44" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="45" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="44" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="45" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="44" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="44" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="45" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="45" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="45" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="46" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="46" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="56" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26587,16 +26598,16 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="43" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="44" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="44" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="44" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="43" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="43" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="42" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -26605,10 +26616,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="42" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="43" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26617,20 +26628,32 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="50" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="51" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="43" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="42" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="42" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="42" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="41" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="56" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="41" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -26638,28 +26661,46 @@
     <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="40" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="39" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="58" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="57" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="38" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="38" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -26668,115 +26709,85 @@
     <xf numFmtId="49" fontId="38" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="38" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="38" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="38" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="38" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="38" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="41" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="58" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="37" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="57" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="57" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="40" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="57" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="36" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="37" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="44" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="36" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="36" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="35" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="43" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="35" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -26785,91 +26796,91 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="44" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="45" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="35" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="34" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="33" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="29" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="38" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="37" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="38" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -26878,7 +26889,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -26890,85 +26901,85 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="39" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="40" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="39" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="40" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="65" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="66" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="25" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="57" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="58" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -26980,55 +26991,58 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="36" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="31" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="30" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -27037,16 +27051,16 @@
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="32" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="33" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -27058,16 +27072,16 @@
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -27086,10 +27100,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -27126,9 +27140,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>3292929</xdr:colOff>
+      <xdr:colOff>3296739</xdr:colOff>
       <xdr:row>333</xdr:row>
-      <xdr:rowOff>2573838</xdr:rowOff>
+      <xdr:rowOff>2570028</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27170,9 +27184,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>3177612</xdr:colOff>
+      <xdr:colOff>3181422</xdr:colOff>
       <xdr:row>413</xdr:row>
-      <xdr:rowOff>1316579</xdr:rowOff>
+      <xdr:rowOff>1312769</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27216,7 +27230,7 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>3429000</xdr:colOff>
       <xdr:row>431</xdr:row>
-      <xdr:rowOff>1696611</xdr:rowOff>
+      <xdr:rowOff>1692801</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27258,9 +27272,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1886547</xdr:colOff>
+      <xdr:colOff>1882737</xdr:colOff>
       <xdr:row>432</xdr:row>
-      <xdr:rowOff>1769588</xdr:rowOff>
+      <xdr:rowOff>1773398</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27302,9 +27316,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>3981355</xdr:colOff>
+      <xdr:colOff>3985165</xdr:colOff>
       <xdr:row>433</xdr:row>
-      <xdr:rowOff>816348</xdr:rowOff>
+      <xdr:rowOff>820158</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27346,9 +27360,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2306502</xdr:colOff>
+      <xdr:colOff>2302692</xdr:colOff>
       <xdr:row>428</xdr:row>
-      <xdr:rowOff>1394326</xdr:rowOff>
+      <xdr:rowOff>1390516</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27390,7 +27404,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>3068974</xdr:colOff>
+      <xdr:colOff>3065164</xdr:colOff>
       <xdr:row>464</xdr:row>
       <xdr:rowOff>1374733</xdr:rowOff>
     </xdr:to>
@@ -27434,9 +27448,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2459066</xdr:colOff>
+      <xdr:colOff>2455256</xdr:colOff>
       <xdr:row>414</xdr:row>
-      <xdr:rowOff>1279609</xdr:rowOff>
+      <xdr:rowOff>1275799</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27478,9 +27492,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>6268301</xdr:colOff>
+      <xdr:colOff>6264491</xdr:colOff>
       <xdr:row>414</xdr:row>
-      <xdr:rowOff>1425173</xdr:rowOff>
+      <xdr:rowOff>1428983</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27522,9 +27536,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2417177</xdr:colOff>
+      <xdr:colOff>2420987</xdr:colOff>
       <xdr:row>414</xdr:row>
-      <xdr:rowOff>854363</xdr:rowOff>
+      <xdr:rowOff>858173</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27566,9 +27580,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2270530</xdr:colOff>
+      <xdr:colOff>2266720</xdr:colOff>
       <xdr:row>458</xdr:row>
-      <xdr:rowOff>972042</xdr:rowOff>
+      <xdr:rowOff>968232</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27612,7 +27626,7 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>3162300</xdr:colOff>
       <xdr:row>512</xdr:row>
-      <xdr:rowOff>2193967</xdr:rowOff>
+      <xdr:rowOff>2190157</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27654,9 +27668,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>6302973</xdr:colOff>
+      <xdr:colOff>6306783</xdr:colOff>
       <xdr:row>512</xdr:row>
-      <xdr:rowOff>1431834</xdr:rowOff>
+      <xdr:rowOff>1428024</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27698,9 +27712,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>3375272</xdr:colOff>
+      <xdr:colOff>3371462</xdr:colOff>
       <xdr:row>614</xdr:row>
-      <xdr:rowOff>2039620</xdr:rowOff>
+      <xdr:rowOff>2035810</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27742,9 +27756,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>4779934</xdr:colOff>
+      <xdr:colOff>4783744</xdr:colOff>
       <xdr:row>614</xdr:row>
-      <xdr:rowOff>893497</xdr:rowOff>
+      <xdr:rowOff>897307</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27786,7 +27800,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>4591166</xdr:colOff>
+      <xdr:colOff>4587356</xdr:colOff>
       <xdr:row>617</xdr:row>
       <xdr:rowOff>917110</xdr:rowOff>
     </xdr:to>
@@ -27830,7 +27844,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>3104027</xdr:colOff>
+      <xdr:colOff>3107837</xdr:colOff>
       <xdr:row>617</xdr:row>
       <xdr:rowOff>2055091</xdr:rowOff>
     </xdr:to>
@@ -27874,7 +27888,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2306502</xdr:colOff>
+      <xdr:colOff>2302692</xdr:colOff>
       <xdr:row>117</xdr:row>
       <xdr:rowOff>1026727</xdr:rowOff>
     </xdr:to>
@@ -27918,9 +27932,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4741971</xdr:colOff>
+      <xdr:colOff>4745781</xdr:colOff>
       <xdr:row>533</xdr:row>
-      <xdr:rowOff>1162850</xdr:rowOff>
+      <xdr:rowOff>1159040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27962,9 +27976,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2343752</xdr:colOff>
+      <xdr:colOff>2339942</xdr:colOff>
       <xdr:row>534</xdr:row>
-      <xdr:rowOff>1198124</xdr:rowOff>
+      <xdr:rowOff>1201934</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -28006,9 +28020,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>6797361</xdr:colOff>
+      <xdr:colOff>6801171</xdr:colOff>
       <xdr:row>535</xdr:row>
-      <xdr:rowOff>1158471</xdr:rowOff>
+      <xdr:rowOff>1162281</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -28050,7 +28064,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2152642</xdr:colOff>
+      <xdr:colOff>2156452</xdr:colOff>
       <xdr:row>536</xdr:row>
       <xdr:rowOff>1180678</xdr:rowOff>
     </xdr:to>
@@ -28094,9 +28108,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2304290</xdr:colOff>
+      <xdr:colOff>2308100</xdr:colOff>
       <xdr:row>537</xdr:row>
-      <xdr:rowOff>1235364</xdr:rowOff>
+      <xdr:rowOff>1239174</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -28138,9 +28152,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4937529</xdr:colOff>
+      <xdr:colOff>4933719</xdr:colOff>
       <xdr:row>544</xdr:row>
-      <xdr:rowOff>1199405</xdr:rowOff>
+      <xdr:rowOff>1203215</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -28184,7 +28198,7 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>2475967</xdr:colOff>
       <xdr:row>545</xdr:row>
-      <xdr:rowOff>1123835</xdr:rowOff>
+      <xdr:rowOff>1127645</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -28226,9 +28240,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4060505</xdr:colOff>
+      <xdr:colOff>4056695</xdr:colOff>
       <xdr:row>546</xdr:row>
-      <xdr:rowOff>1163522</xdr:rowOff>
+      <xdr:rowOff>1159712</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -28270,9 +28284,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2649276</xdr:colOff>
+      <xdr:colOff>2645466</xdr:colOff>
       <xdr:row>539</xdr:row>
-      <xdr:rowOff>1197403</xdr:rowOff>
+      <xdr:rowOff>1201213</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -28314,9 +28328,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>4250803</xdr:colOff>
+      <xdr:colOff>4246993</xdr:colOff>
       <xdr:row>539</xdr:row>
-      <xdr:rowOff>1539471</xdr:rowOff>
+      <xdr:rowOff>1543281</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -28358,9 +28372,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>4359300</xdr:colOff>
+      <xdr:colOff>4363110</xdr:colOff>
       <xdr:row>537</xdr:row>
-      <xdr:rowOff>1238338</xdr:rowOff>
+      <xdr:rowOff>1234528</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -28849,29 +28863,34 @@
         <v>17</v>
       </c>
     </row>
+    <row r="11" spans="1:22">
+      <c r="A11" s="10" t="s">
+        <v>1398</v>
+      </c>
+    </row>
     <row r="12" spans="1:22" ht="244.8">
       <c r="A12" s="1" t="s">
         <v>1392</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1394</v>
-      </c>
-      <c r="C12" s="275" t="s">
         <v>1393</v>
       </c>
+      <c r="C12" s="276" t="s">
+        <v>1397</v>
+      </c>
       <c r="D12" s="275" t="s">
-        <v>1397</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="216">
       <c r="A13" s="1" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C13" s="275" t="s">
+        <v>1394</v>
+      </c>
+      <c r="D13" s="275" t="s">
         <v>1396</v>
-      </c>
-      <c r="C13" s="275" t="s">
-        <v>1395</v>
-      </c>
-      <c r="D13" s="275" t="s">
-        <v>1397</v>
       </c>
     </row>
     <row r="16" spans="1:22">
@@ -35344,7 +35363,7 @@
       <c r="D675" s="31"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="56" type="noConversion"/>
+  <phoneticPr fontId="57" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D273" r:id="rId1" xr:uid="{86D65E8A-CF7A-4E7D-9853-37328E3CAC93}"/>
   </hyperlinks>

</xml_diff>